<commit_message>
docs(planning): mark 4 catalog management features as delivered
Updates rows 20–23 of Avanzamento tool Niuexa new.xlsx:
- Aggiornamenti in Massa delle Liste di Prodotti: 🔴 → 🟢
- Gestione dei Prezzi: 🔴 → 🟢
- Aggiornamenti sulla Disponibilità/Inventario: 🔴 → 🟢
- Gestione delle Immagini: 🔴 → 🟢

The "Note" column on each row is replaced with a technical summary
(endpoints, validation, audit log table, test files, UX behavior)
matching the convention used by other 🟢 rows.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/planning/Avanzamento tool Niuexa new.xlsx
+++ b/docs/planning/Avanzamento tool Niuexa new.xlsx
@@ -1013,12 +1013,12 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟢</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Da preview non è ancora integrata funzionalità</t>
+          <t>POST /catalog/bulk-update accetta Excel e ritorna BulkResult{successes,errors} con codice errore per riga (sp_api_error, invalid_input, ecc.). Audit log persistito su tabella catalog_change_log. Test backend/tests/test_catalog_service.py copre mix successo/fallimento. UI BulkUpdateCard mostra tabella per-row + conferma esplicita prima del submit.</t>
         </is>
       </c>
       <c r="F20" s="2" t="n"/>
@@ -1041,12 +1041,12 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟢</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Da preview non è ancora integrata funzionalità</t>
+          <t>POST /catalog/prices con validazione Pydantic (Decimal&gt;=0, ASIN regex, currency 3-letter) e Zod nel frontend. Ritorna BulkResult[PriceUpdateResult]. Conferma esplicita prima del submit; tabella risultati con badge OK/Failed per riga. History per ASIN via GET /catalog/products/{asin}/history.</t>
         </is>
       </c>
       <c r="F21" s="2" t="n"/>
@@ -1069,12 +1069,12 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟢</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Da preview non è ancora integrata funzionalità</t>
+          <t>PATCH /catalog/products/{asin}/availability con quantity opzionale (&gt;=0). Mirror locale + SP-API set_listing_quantity; fallimento SP-API registrato comunque su catalog_change_log. UI: conferma esplicita per disable (destructive); Zod valida ASIN format prima del submit.</t>
         </is>
       </c>
       <c r="F22" s="2" t="n"/>
@@ -1097,12 +1097,12 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟢</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Da preview non è ancora integrata funzionalità</t>
+          <t>POST /catalog/products/{asin}/images con validazione MIME (jpeg/png/webp) e cap 10MB (Pydantic + Zod client-side). S3 prefisso tenant-scoped catalog/{org}/{account}/{asin}/. SP-API patch via update_listing_images (main + 8 alt). Audit log scrive anche su fallimento SP-API; UI separa sp_api_error in banner dedicato.</t>
         </is>
       </c>
       <c r="F23" s="2" t="n"/>

</xml_diff>

<commit_message>
docs(planning): mark item 10 (data retention) as delivered
Particionamento automatizzato — migration 023_partition_ts_tables (in PR #1)
converts sales_data, advertising_metrics, advertising_metrics_by_asin,
bsr_history to PARTITION BY RANGE (date). manage_partitions cron auto-creates
N+1/N+2 monthly partitions and drops those beyond DATA_RETENTION_MONTHS.

Item 10 was the last 🟡 caused by internal tech debt — moves to 🟢 once both
PRs are merged. The 6 remaining 🟡 are all externally blocked (SendGrid key,
Amazon Ads OAuth, real client names, forecast realism PM decision).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/planning/Avanzamento tool Niuexa new.xlsx
+++ b/docs/planning/Avanzamento tool Niuexa new.xlsx
@@ -749,19 +749,15 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>DATA_RETENTION_MONTHS=24 + manage_data_retention task con VACUUM ANALYZE. manage_partitions resta operativo; ripartizionamenti rischiosi vanno eseguiti manualmente.</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Non ancora presente</t>
-        </is>
-      </c>
+          <t>Particionamento automatizzato via migration 023_partition_ts_tables (sales_data, advertising_metrics, advertising_metrics_by_asin, bsr_history) con PK composta (id, date). workers/tasks/maintenance.py::manage_partitions auto-crea partizioni N+1/N+2 via UDF ensure_monthly_partition e droppa quelle outside DATA_RETENTION_MONTHS (24). Ripartizionamenti DDL idempotenti — niente più operazioni manuali rischiose. Migration 023 prende ACCESS EXCLUSIVE LOCK durante la conversione iniziale: eseguire in maintenance window con API+workers fermi.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">

</xml_diff>